<commit_message>
Added a few color details
</commit_message>
<xml_diff>
--- a/BambuFilamentList.xlsx
+++ b/BambuFilamentList.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/75293e77613b4537/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dragon\repos\bambu-tag-parsing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2036" documentId="8_{8F966C42-446D-4962-8A3C-C0E9B49B6882}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{818C7120-E7E0-4969-A9ED-1B7FCF8E1264}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A304F1EB-31C3-4ECD-B1C7-758EDFE298D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{D89A2817-7CF1-4374-82CB-88050B4D4E91}"/>
+    <workbookView xWindow="-38520" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{D89A2817-7CF1-4374-82CB-88050B4D4E91}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1738" uniqueCount="613">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1746" uniqueCount="621">
   <si>
     <t>FilamentType</t>
   </si>
@@ -1875,6 +1875,30 @@
   </si>
   <si>
     <t>GFS06</t>
+  </si>
+  <si>
+    <t>A10-W0</t>
+  </si>
+  <si>
+    <t>A10-D1</t>
+  </si>
+  <si>
+    <t>GFA10</t>
+  </si>
+  <si>
+    <t>A17-P1</t>
+  </si>
+  <si>
+    <t>B8ACD680</t>
+  </si>
+  <si>
+    <t>959698FF</t>
+  </si>
+  <si>
+    <t>A10-B0</t>
+  </si>
+  <si>
+    <t>009BD8FF</t>
   </si>
 </sst>
 </file>
@@ -1944,10 +1968,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -8673,8 +8693,13 @@
       <c r="E113">
         <v>13711</v>
       </c>
-      <c r="F113"/>
+      <c r="F113" t="s">
+        <v>617</v>
+      </c>
       <c r="G113"/>
+      <c r="H113" t="s">
+        <v>616</v>
+      </c>
       <c r="I113" t="s">
         <v>248</v>
       </c>
@@ -8728,7 +8753,7 @@
       <c r="F114"/>
       <c r="G114"/>
       <c r="I114" t="s">
-        <v>248</v>
+        <v>615</v>
       </c>
       <c r="J114" t="s">
         <v>221</v>
@@ -8777,10 +8802,15 @@
       <c r="E115">
         <v>12107</v>
       </c>
-      <c r="F115"/>
+      <c r="F115" t="s">
+        <v>217</v>
+      </c>
       <c r="G115"/>
+      <c r="H115" t="s">
+        <v>613</v>
+      </c>
       <c r="I115" t="s">
-        <v>248</v>
+        <v>615</v>
       </c>
       <c r="J115" t="s">
         <v>221</v>
@@ -8832,7 +8862,7 @@
       <c r="F116"/>
       <c r="G116"/>
       <c r="I116" t="s">
-        <v>248</v>
+        <v>615</v>
       </c>
       <c r="J116" t="s">
         <v>221</v>
@@ -8889,7 +8919,7 @@
         <v>458</v>
       </c>
       <c r="I117" t="s">
-        <v>248</v>
+        <v>615</v>
       </c>
       <c r="J117" t="s">
         <v>221</v>
@@ -8941,7 +8971,7 @@
       <c r="F118"/>
       <c r="G118"/>
       <c r="I118" t="s">
-        <v>248</v>
+        <v>615</v>
       </c>
       <c r="J118" t="s">
         <v>221</v>
@@ -8990,10 +9020,15 @@
       <c r="E119">
         <v>12106</v>
       </c>
-      <c r="F119"/>
+      <c r="F119" t="s">
+        <v>618</v>
+      </c>
       <c r="G119"/>
+      <c r="H119" t="s">
+        <v>614</v>
+      </c>
       <c r="I119" t="s">
-        <v>248</v>
+        <v>615</v>
       </c>
       <c r="J119" t="s">
         <v>221</v>
@@ -9042,10 +9077,15 @@
       <c r="E120">
         <v>12601</v>
       </c>
-      <c r="F120"/>
+      <c r="F120" t="s">
+        <v>620</v>
+      </c>
       <c r="G120"/>
+      <c r="H120" t="s">
+        <v>619</v>
+      </c>
       <c r="I120" t="s">
-        <v>248</v>
+        <v>615</v>
       </c>
       <c r="J120" t="s">
         <v>221</v>

</xml_diff>